<commit_message>
Fix the Worked example sheet in the PERT workbook
The six chapter activities were missing their description field, so every
value sat one column to the left and b was blank. Paths header shortened so
it no longer wraps.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/week-07-pert-studio.xlsx
+++ b/files/week-07-pert-studio.xlsx
@@ -661,16 +661,21 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
+          <t>Activity A</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>47</v>
       </c>
       <c r="G5" s="6" t="n"/>
@@ -690,16 +695,21 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
+          <t>Activity B</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="E6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="G6" s="6" t="n"/>
@@ -719,16 +729,21 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
+          <t>Activity C</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>28</v>
       </c>
       <c r="G7" s="6" t="n"/>
@@ -748,16 +763,21 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
+          <t>Activity D</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="D8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="G8" s="6" t="n"/>
@@ -777,16 +797,21 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
+          <t>Activity E</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="D9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>14</v>
       </c>
       <c r="G9" s="6" t="n"/>
@@ -806,16 +831,21 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
+          <t>Activity F</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
           <t>D, E</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="D10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="E10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="G10" s="6" t="n"/>
@@ -844,12 +874,12 @@
       <c r="C13" s="11" t="n"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Sum t_e</t>
+          <t>Σ t_e</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Sum variance</t>
+          <t>Σ var</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -857,14 +887,6 @@
           <t>σ</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
-      <c r="N13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -1353,12 +1375,12 @@
       <c r="C14" s="11" t="n"/>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Sum t_e</t>
+          <t>Σ t_e</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Sum variance</t>
+          <t>Σ var</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1366,14 +1388,6 @@
           <t>σ</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
-      <c r="N14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Publish site (gated as of build date) 29fafffce5a316a8dabcc8b16318363d90e2c535
</commit_message>
<xml_diff>
--- a/files/week-07-pert-studio.xlsx
+++ b/files/week-07-pert-studio.xlsx
@@ -661,16 +661,21 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
+          <t>Activity A</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>47</v>
       </c>
       <c r="G5" s="6" t="n"/>
@@ -690,16 +695,21 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
+          <t>Activity B</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="E6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="G6" s="6" t="n"/>
@@ -719,16 +729,21 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
+          <t>Activity C</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>28</v>
       </c>
       <c r="G7" s="6" t="n"/>
@@ -748,16 +763,21 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
+          <t>Activity D</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="D8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="G8" s="6" t="n"/>
@@ -777,16 +797,21 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
+          <t>Activity E</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="D9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>14</v>
       </c>
       <c r="G9" s="6" t="n"/>
@@ -806,16 +831,21 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
+          <t>Activity F</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
           <t>D, E</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="D10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="E10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="G10" s="6" t="n"/>
@@ -844,12 +874,12 @@
       <c r="C13" s="11" t="n"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Sum t_e</t>
+          <t>Σ t_e</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Sum variance</t>
+          <t>Σ var</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -857,14 +887,6 @@
           <t>σ</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
-      <c r="N13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -1353,12 +1375,12 @@
       <c r="C14" s="11" t="n"/>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Sum t_e</t>
+          <t>Σ t_e</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Sum variance</t>
+          <t>Σ var</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1366,14 +1388,6 @@
           <t>σ</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
-      <c r="N14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>